<commit_message>
test: rename demo attendee to Adarsh and verify submission compliance
</commit_message>
<xml_diff>
--- a/agents/event-networking-matchmaker/sample/form-responses.xlsx
+++ b/agents/event-networking-matchmaker/sample/form-responses.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form Responses 1" sheetId="1" r:id="Red9b74e085194977"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form Responses 1" sheetId="1" r:id="R8280a7f7f460466f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -328,7 +328,7 @@
         <x:v>P001</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
-        <x:v>Arun</x:v>
+        <x:v>Adarsh</x:v>
       </x:c>
       <x:c r="C2" s="3" t="str">
         <x:v>Python, API</x:v>
@@ -849,7 +849,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7abe0b19834941b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b51ad629fd54af2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>